<commit_message>
new SW version Aug 11, 2026, replace web-conole/data with data_sample
</commit_message>
<xml_diff>
--- a/web-console/server/assets/excel_template.xlsx
+++ b/web-console/server/assets/excel_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\DEV\UBA6\web-console\server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23D716DC-4133-4304-A888-8D23E37D970E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93D08DA2-7AC9-470B-A1E0-87F197B9FB35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3E3B58E4-0181-4207-8002-E1D914CEBC2E}"/>
   </bookViews>
   <sheets>
     <sheet name="Report" sheetId="1" r:id="rId1"/>
@@ -407,8 +407,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFCC0000"/>
       <color rgb="FF000000"/>
-      <color rgb="FFCC0000"/>
       <color rgb="FF009999"/>
       <color rgb="FF0066FF"/>
       <color rgb="FF009900"/>
@@ -1544,25 +1544,19 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Data!$A$2:$A$50000</c:f>
+              <c:f>Data!$K$2:$K$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Data!$E$2:$E$50000</c:f>
+              <c:f>Data!$N$2:$N$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -2423,7 +2417,7 @@
           <c:spPr>
             <a:ln w="12700" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="tx1"/>
+                <a:schemeClr val="accent6"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -2434,25 +2428,19 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Data!$A$2:$A$50000</c:f>
+              <c:f>Data!$K$2:$K$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Data!$C$2:$C$50000</c:f>
+              <c:f>Data!$L$2:$L$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -2546,9 +2534,9 @@
                   <c:v>Voltage [V]</c:v>
                 </c:tx>
                 <c:spPr>
-                  <a:ln w="15875" cap="rnd">
+                  <a:ln w="12700" cap="rnd">
                     <a:solidFill>
-                      <a:schemeClr val="accent1"/>
+                      <a:schemeClr val="tx1"/>
                     </a:solidFill>
                     <a:round/>
                   </a:ln>
@@ -2690,25 +2678,19 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Data!$A$2:$A$50000</c:f>
+              <c:f>Data!$K$2:$K$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Data!$D$2:$D$50000</c:f>
+              <c:f>Data!$M$2:$M$50000</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="49999"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -3019,9 +3001,11 @@
   </c:chart>
   <c:spPr>
     <a:solidFill>
-      <a:srgbClr val="000000">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="50000"/>
+        <a:lumOff val="50000"/>
         <a:alpha val="0"/>
-      </a:srgbClr>
+      </a:schemeClr>
     </a:solidFill>
     <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:noFill/>
@@ -5929,13 +5913,13 @@
       <xdr:col>1</xdr:col>
       <xdr:colOff>110620</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>97678</xdr:rowOff>
+      <xdr:rowOff>85364</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>92735</xdr:colOff>
+      <xdr:colOff>96545</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>82976</xdr:rowOff>
+      <xdr:rowOff>76377</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -5950,8 +5934,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="620888" y="390232"/>
-          <a:ext cx="9275793" cy="4271548"/>
+          <a:off x="620888" y="367916"/>
+          <a:ext cx="9320017" cy="4156296"/>
           <a:chOff x="621310" y="383428"/>
           <a:chExt cx="9321752" cy="4231579"/>
         </a:xfrm>

</xml_diff>